<commit_message>
Fix XLSForm structure + regenerate bulk-upload files
- data/form-template.xlsx: rebuild to valid XLSForm structure. Three sheets
  (survey/choices/settings) with column headers as row 1; no literal
  'survey'/'choices'/'settings' marker cells (Kobo's strict deploy path was
  rejecting the prior version that had section names as data).
- data/feedback.xlsx: regenerate from data/feedback.jsonl with snake_case
  'name'-attribute columns matching the form-template schema (date,
  feedback_channel, is_emergency, gender, etc.). Categorical values are
  normalized to choice slugs; Kobo-internal metadata columns (_id/_uuid/
  _submission_time) are stripped.
- data/feedback.jsonl: include name-keyed JSONL records for OpenRosa XML
  programmatic ingestion (one JSON object per line).
- README.md: clarify the structure distinction between form-template.*
  (questions/schema) and feedback.* (records/answers) so the two
  upload paths (Replace-with-XLSForm vs Replace data) aren't conflated.
</commit_message>
<xml_diff>
--- a/data/form-template.xlsx
+++ b/data/form-template.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,23 +27,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00403833"/>
-        <bgColor rgb="00403833"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -58,11 +48,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,30 +417,24 @@
   </sheetPr>
   <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>required</t>
         </is>
@@ -956,24 +937,19 @@
   </sheetPr>
   <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>list_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
@@ -1230,24 +1206,19 @@
   </sheetPr>
   <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="33" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>form_title</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>form_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>version</t>
         </is>

</xml_diff>